<commit_message>
Oatside report: publish reports/oatside-pg-2026 (remove legacy oatside-apr2026) 2026-05-05 14:39
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customer_Summary'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Customer_Trips_Per_Day'!$A$1:$C$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit_Log'!$A$1:$J$70</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$W$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$Z$106</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Unmatched_Log'!$A$1:$H$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Daily_Activity'!$A$1:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$73</definedName>
@@ -531,7 +531,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05 12:56</t>
+          <t>2026-05-05 14:39</t>
         </is>
       </c>
     </row>
@@ -6257,7 +6257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W106"/>
+  <dimension ref="A1:Z106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6281,8 +6281,11 @@
     <col width="24" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="15" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6393,10 +6396,25 @@
       </c>
       <c r="V1" s="4" t="inlineStr">
         <is>
+          <t>Trip_rate_baht</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>Downtime_50_baht</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>Downtime_100_baht</t>
+        </is>
+      </c>
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
           <t>Nw_outbound50_baht</t>
         </is>
       </c>
-      <c r="W1" s="4" t="inlineStr">
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>Return_manual_baht</t>
         </is>
@@ -6475,9 +6493,18 @@
         <v>1</v>
       </c>
       <c r="V2" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6554,9 +6581,18 @@
         <v>1</v>
       </c>
       <c r="V3" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6633,9 +6669,18 @@
         <v>1</v>
       </c>
       <c r="V4" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6712,9 +6757,18 @@
         <v>1</v>
       </c>
       <c r="V5" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6791,9 +6845,18 @@
         <v>1</v>
       </c>
       <c r="V6" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6874,9 +6937,18 @@
         <v>1</v>
       </c>
       <c r="V7" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6953,9 +7025,18 @@
         <v>1</v>
       </c>
       <c r="V8" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7032,9 +7113,18 @@
         <v>1</v>
       </c>
       <c r="V9" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7111,9 +7201,18 @@
         <v>1</v>
       </c>
       <c r="V10" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W10" s="6" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7190,9 +7289,18 @@
         <v>1</v>
       </c>
       <c r="V11" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W11" s="7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7269,9 +7377,18 @@
         <v>1</v>
       </c>
       <c r="V12" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7348,9 +7465,18 @@
         <v>1</v>
       </c>
       <c r="V13" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7427,9 +7553,18 @@
         <v>1</v>
       </c>
       <c r="V14" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7506,9 +7641,18 @@
         <v>1</v>
       </c>
       <c r="V15" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W15" s="7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7585,9 +7729,18 @@
         <v>1</v>
       </c>
       <c r="V16" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W16" s="6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7664,9 +7817,18 @@
         <v>1</v>
       </c>
       <c r="V17" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7743,9 +7905,18 @@
         <v>1</v>
       </c>
       <c r="V18" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7822,9 +7993,18 @@
         <v>1</v>
       </c>
       <c r="V19" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W19" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7901,9 +8081,18 @@
         <v>1</v>
       </c>
       <c r="V20" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W20" s="6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7980,9 +8169,18 @@
         <v>1</v>
       </c>
       <c r="V21" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W21" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8059,9 +8257,18 @@
         <v>1</v>
       </c>
       <c r="V22" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W22" s="6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8138,9 +8345,18 @@
         <v>1</v>
       </c>
       <c r="V23" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W23" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8217,9 +8433,18 @@
         <v>1</v>
       </c>
       <c r="V24" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8296,9 +8521,18 @@
         <v>1</v>
       </c>
       <c r="V25" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8375,9 +8609,18 @@
         <v>1</v>
       </c>
       <c r="V26" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W26" s="6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z26" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8454,9 +8697,18 @@
         <v>1</v>
       </c>
       <c r="V27" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W27" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8533,9 +8785,18 @@
         <v>1</v>
       </c>
       <c r="V28" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8612,9 +8873,18 @@
         <v>1</v>
       </c>
       <c r="V29" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W29" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8691,9 +8961,18 @@
         <v>1</v>
       </c>
       <c r="V30" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8770,9 +9049,18 @@
         <v>1</v>
       </c>
       <c r="V31" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8849,9 +9137,18 @@
         <v>1</v>
       </c>
       <c r="V32" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z32" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8932,9 +9229,18 @@
         <v>1</v>
       </c>
       <c r="V33" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W33" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X33" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y33" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z33" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9011,9 +9317,18 @@
         <v>1</v>
       </c>
       <c r="V34" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z34" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9090,9 +9405,18 @@
         <v>1</v>
       </c>
       <c r="V35" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9169,9 +9493,18 @@
         <v>1</v>
       </c>
       <c r="V36" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9248,9 +9581,18 @@
         <v>1</v>
       </c>
       <c r="V37" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9327,9 +9669,18 @@
         <v>1</v>
       </c>
       <c r="V38" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z38" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9406,9 +9757,18 @@
         <v>1</v>
       </c>
       <c r="V39" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W39" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9485,9 +9845,18 @@
         <v>1</v>
       </c>
       <c r="V40" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W40" s="6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z40" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9564,9 +9933,18 @@
         <v>1</v>
       </c>
       <c r="V41" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z41" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9643,9 +10021,18 @@
         <v>1</v>
       </c>
       <c r="V42" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9722,9 +10109,18 @@
         <v>1</v>
       </c>
       <c r="V43" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W43" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X43" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y43" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z43" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9801,9 +10197,18 @@
         <v>1</v>
       </c>
       <c r="V44" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z44" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9880,9 +10285,18 @@
         <v>1</v>
       </c>
       <c r="V45" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W45" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X45" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y45" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z45" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9959,9 +10373,18 @@
         <v>1</v>
       </c>
       <c r="V46" s="6" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z46" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10038,9 +10461,18 @@
         <v>1</v>
       </c>
       <c r="V47" s="7" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="W47" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="X47" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y47" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z47" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10117,9 +10549,18 @@
         <v>1</v>
       </c>
       <c r="V48" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z48" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10196,9 +10637,18 @@
         <v>1</v>
       </c>
       <c r="V49" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W49" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X49" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y49" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z49" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10279,9 +10729,18 @@
         <v>1</v>
       </c>
       <c r="V50" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W50" s="6" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X50" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y50" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z50" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10358,9 +10817,18 @@
         <v>1</v>
       </c>
       <c r="V51" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W51" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X51" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y51" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z51" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10437,9 +10905,18 @@
         <v>1</v>
       </c>
       <c r="V52" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W52" s="6" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z52" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10516,9 +10993,18 @@
         <v>1</v>
       </c>
       <c r="V53" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W53" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X53" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y53" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z53" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10595,9 +11081,18 @@
         <v>1</v>
       </c>
       <c r="V54" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z54" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10674,9 +11169,18 @@
         <v>1</v>
       </c>
       <c r="V55" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W55" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X55" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y55" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z55" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10753,9 +11257,18 @@
         <v>1</v>
       </c>
       <c r="V56" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y56" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z56" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10832,9 +11345,18 @@
         <v>1</v>
       </c>
       <c r="V57" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W57" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X57" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y57" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z57" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10911,9 +11433,18 @@
         <v>1</v>
       </c>
       <c r="V58" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z58" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10990,9 +11521,18 @@
         <v>1</v>
       </c>
       <c r="V59" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W59" s="7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X59" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y59" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z59" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11069,9 +11609,18 @@
         <v>1</v>
       </c>
       <c r="V60" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W60" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X60" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y60" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z60" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11152,9 +11701,18 @@
         <v>1</v>
       </c>
       <c r="V61" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W61" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X61" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y61" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z61" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11231,9 +11789,18 @@
         <v>1</v>
       </c>
       <c r="V62" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W62" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X62" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y62" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z62" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11310,9 +11877,18 @@
         <v>1</v>
       </c>
       <c r="V63" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W63" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X63" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y63" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z63" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11389,9 +11965,18 @@
         <v>1</v>
       </c>
       <c r="V64" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W64" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X64" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y64" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z64" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11468,9 +12053,18 @@
         <v>1</v>
       </c>
       <c r="V65" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W65" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X65" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y65" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z65" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11547,9 +12141,18 @@
         <v>1</v>
       </c>
       <c r="V66" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W66" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X66" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y66" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z66" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11630,9 +12233,18 @@
         <v>1</v>
       </c>
       <c r="V67" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z67" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11709,9 +12321,18 @@
         <v>1</v>
       </c>
       <c r="V68" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W68" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X68" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y68" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z68" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11788,9 +12409,18 @@
         <v>1</v>
       </c>
       <c r="V69" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W69" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X69" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y69" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z69" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11867,9 +12497,18 @@
         <v>1</v>
       </c>
       <c r="V70" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W70" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X70" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y70" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z70" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11946,9 +12585,18 @@
         <v>1</v>
       </c>
       <c r="V71" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W71" s="7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X71" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y71" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z71" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12025,9 +12673,18 @@
         <v>1</v>
       </c>
       <c r="V72" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W72" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X72" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y72" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z72" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12104,9 +12761,18 @@
         <v>1</v>
       </c>
       <c r="V73" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z73" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12183,9 +12849,18 @@
         <v>1</v>
       </c>
       <c r="V74" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W74" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X74" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y74" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z74" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12266,9 +12941,18 @@
         <v>1</v>
       </c>
       <c r="V75" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z75" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12345,9 +13029,18 @@
         <v>1</v>
       </c>
       <c r="V76" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W76" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X76" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y76" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z76" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12424,9 +13117,18 @@
         <v>1</v>
       </c>
       <c r="V77" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W77" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X77" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y77" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z77" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12507,9 +13209,18 @@
         <v>1</v>
       </c>
       <c r="V78" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W78" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X78" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y78" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z78" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12586,9 +13297,18 @@
         <v>1</v>
       </c>
       <c r="V79" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z79" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12665,9 +13385,18 @@
         <v>1</v>
       </c>
       <c r="V80" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W80" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X80" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y80" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z80" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12748,9 +13477,18 @@
         <v>1</v>
       </c>
       <c r="V81" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W81" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X81" s="7" t="n">
+        <v>7500</v>
+      </c>
+      <c r="Y81" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12827,9 +13565,18 @@
         <v>1</v>
       </c>
       <c r="V82" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W82" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X82" s="6" t="n">
+        <v>7500</v>
+      </c>
+      <c r="Y82" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z82" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12906,9 +13653,18 @@
         <v>1</v>
       </c>
       <c r="V83" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W83" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X83" s="7" t="n">
+        <v>7500</v>
+      </c>
+      <c r="Y83" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z83" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12985,9 +13741,18 @@
         <v>1</v>
       </c>
       <c r="V84" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W84" s="6" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y84" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z84" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13064,9 +13829,18 @@
         <v>1</v>
       </c>
       <c r="V85" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W85" s="7" t="n">
+        <v>7500</v>
+      </c>
+      <c r="X85" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y85" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z85" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13143,9 +13917,18 @@
         <v>1</v>
       </c>
       <c r="V86" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W86" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X86" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y86" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z86" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13222,9 +14005,18 @@
         <v>1</v>
       </c>
       <c r="V87" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W87" s="7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X87" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y87" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z87" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13301,9 +14093,18 @@
         <v>1</v>
       </c>
       <c r="V88" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W88" s="6" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y88" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z88" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13380,9 +14181,18 @@
         <v>1</v>
       </c>
       <c r="V89" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W89" s="7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X89" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y89" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z89" s="7" t="n">
         <v>7500</v>
       </c>
     </row>
@@ -13459,9 +14269,18 @@
         <v>1</v>
       </c>
       <c r="V90" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W90" s="6" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X90" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y90" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z90" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13538,9 +14357,18 @@
         <v>1</v>
       </c>
       <c r="V91" s="7" t="n">
+        <v>7500</v>
+      </c>
+      <c r="W91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y91" s="7" t="n">
         <v>3750</v>
       </c>
-      <c r="W91" s="7" t="n">
+      <c r="Z91" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13617,9 +14445,18 @@
         <v>1</v>
       </c>
       <c r="V92" s="6" t="n">
+        <v>7500</v>
+      </c>
+      <c r="W92" s="6" t="n">
         <v>3750</v>
       </c>
-      <c r="W92" s="6" t="n">
+      <c r="X92" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y92" s="6" t="n">
+        <v>3750</v>
+      </c>
+      <c r="Z92" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13696,9 +14533,18 @@
         <v>1</v>
       </c>
       <c r="V93" s="7" t="n">
+        <v>7500</v>
+      </c>
+      <c r="W93" s="7" t="n">
         <v>3750</v>
       </c>
-      <c r="W93" s="7" t="n">
+      <c r="X93" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y93" s="7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="Z93" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13775,9 +14621,18 @@
         <v>1</v>
       </c>
       <c r="V94" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W94" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X94" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y94" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z94" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13854,9 +14709,18 @@
         <v>1</v>
       </c>
       <c r="V95" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W95" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X95" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y95" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z95" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13933,9 +14797,18 @@
         <v>1</v>
       </c>
       <c r="V96" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W96" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X96" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y96" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z96" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14012,9 +14885,18 @@
         <v>1</v>
       </c>
       <c r="V97" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W97" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X97" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y97" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z97" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14091,9 +14973,18 @@
         <v>1</v>
       </c>
       <c r="V98" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W98" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X98" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y98" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z98" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14174,9 +15065,18 @@
         <v>1</v>
       </c>
       <c r="V99" s="7" t="n">
+        <v>7500</v>
+      </c>
+      <c r="W99" s="7" t="n">
         <v>3750</v>
       </c>
-      <c r="W99" s="7" t="n">
+      <c r="X99" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y99" s="7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="Z99" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14253,9 +15153,18 @@
         <v>1</v>
       </c>
       <c r="V100" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W100" s="6" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X100" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y100" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z100" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14332,9 +15241,18 @@
         <v>1</v>
       </c>
       <c r="V101" s="7" t="n">
+        <v>7500</v>
+      </c>
+      <c r="W101" s="7" t="n">
         <v>3750</v>
       </c>
-      <c r="W101" s="7" t="n">
+      <c r="X101" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y101" s="7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="Z101" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14411,9 +15329,18 @@
         <v>1</v>
       </c>
       <c r="V102" s="6" t="n">
+        <v>7500</v>
+      </c>
+      <c r="W102" s="6" t="n">
         <v>3750</v>
       </c>
-      <c r="W102" s="6" t="n">
+      <c r="X102" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y102" s="6" t="n">
+        <v>3750</v>
+      </c>
+      <c r="Z102" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14490,9 +15417,18 @@
         <v>1</v>
       </c>
       <c r="V103" s="7" t="n">
+        <v>7500</v>
+      </c>
+      <c r="W103" s="7" t="n">
         <v>3750</v>
       </c>
-      <c r="W103" s="7" t="n">
+      <c r="X103" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y103" s="7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="Z103" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14569,9 +15505,18 @@
         <v>1</v>
       </c>
       <c r="V104" s="6" t="n">
+        <v>7500</v>
+      </c>
+      <c r="W104" s="6" t="n">
         <v>3750</v>
       </c>
-      <c r="W104" s="6" t="n">
+      <c r="X104" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y104" s="6" t="n">
+        <v>3750</v>
+      </c>
+      <c r="Z104" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14648,9 +15593,18 @@
         <v>1</v>
       </c>
       <c r="V105" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W105" s="7" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y105" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z105" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14727,14 +15681,23 @@
         <v>1</v>
       </c>
       <c r="V106" s="6" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="W106" s="6" t="n">
+        <v>3750</v>
+      </c>
+      <c r="X106" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y106" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z106" s="6" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W106"/>
+  <autoFilter ref="A1:Z106"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>